<commit_message>
STX missing small boys
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/ALFA.ST.xlsx
+++ b/data/stx_xlsx/ALFA.ST.xlsx
@@ -855,7 +855,7 @@
     <t>Equipment, tools and installations, Depr</t>
   </si>
   <si>
-    <t>Property,Plant And Equipment, Net - Balancing value</t>
+    <t>Property,Plant And Equipment, Net</t>
   </si>
   <si>
     <t>Other non-current assets</t>
@@ -15046,44 +15046,85 @@
       <c r="W92" s="15"/>
     </row>
     <row r="93" ht="15.0" customHeight="1">
-      <c r="A93" s="14" t="s">
+      <c r="A93" s="27" t="s">
         <v>278</v>
       </c>
       <c r="B93" s="15"/>
-      <c r="C93" s="15"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="15"/>
-      <c r="F93" s="15"/>
-      <c r="G93" s="15"/>
-      <c r="H93" s="15"/>
-      <c r="I93" s="15"/>
-      <c r="J93" s="15"/>
-      <c r="K93" s="15"/>
-      <c r="L93" s="15"/>
-      <c r="M93" s="15"/>
-      <c r="N93" s="15"/>
-      <c r="O93" s="15"/>
-      <c r="P93" s="15"/>
+      <c r="C93" s="15">
+        <f t="shared" ref="C93:H93" si="1">C84+C74+C71+C68</f>
+        <v>11939.27</v>
+      </c>
+      <c r="D93" s="15">
+        <f t="shared" si="1"/>
+        <v>9376</v>
+      </c>
+      <c r="E93" s="15">
+        <f t="shared" si="1"/>
+        <v>7700.5</v>
+      </c>
+      <c r="F93" s="15">
+        <f t="shared" si="1"/>
+        <v>6577.35</v>
+      </c>
+      <c r="G93" s="15">
+        <f t="shared" si="1"/>
+        <v>6441.67</v>
+      </c>
+      <c r="H93" s="15">
+        <f t="shared" si="1"/>
+        <v>5869.77</v>
+      </c>
+      <c r="I93" s="15">
+        <f t="shared" ref="I93:N93" si="2">I84+I74+I71+I68+I91+I92</f>
+        <v>5470.67</v>
+      </c>
+      <c r="J93" s="15">
+        <f t="shared" si="2"/>
+        <v>5295.42</v>
+      </c>
+      <c r="K93" s="15">
+        <f t="shared" si="2"/>
+        <v>5110.48</v>
+      </c>
+      <c r="L93" s="15">
+        <f t="shared" si="2"/>
+        <v>5489.23</v>
+      </c>
+      <c r="M93" s="15">
+        <f t="shared" si="2"/>
+        <v>5256.42</v>
+      </c>
+      <c r="N93" s="15">
+        <f t="shared" si="2"/>
+        <v>3969.62</v>
+      </c>
+      <c r="O93" s="18">
+        <v>3263.19</v>
+      </c>
+      <c r="P93" s="15">
+        <f>P84+P74+P71+P68</f>
+        <v>1910.69</v>
+      </c>
       <c r="Q93" s="18">
-        <v>2903.18</v>
+        <v>3047.21</v>
       </c>
       <c r="R93" s="18">
-        <v>2759.07</v>
+        <v>2870.73</v>
       </c>
       <c r="S93" s="18">
-        <v>2780.61</v>
+        <v>3153.2</v>
       </c>
       <c r="T93" s="18">
-        <v>2111.75</v>
+        <v>2374.98</v>
       </c>
       <c r="U93" s="18">
-        <v>2147.29</v>
+        <v>2289.96</v>
       </c>
       <c r="V93" s="18">
-        <v>2062.52</v>
+        <v>2167.73</v>
       </c>
       <c r="W93" s="18">
-        <v>2108.45</v>
+        <v>2265.46</v>
       </c>
     </row>
     <row r="94" ht="15.0" customHeight="1">

</xml_diff>